<commit_message>
fix(gstr1): omit csamt in b2cl and b2cla when the cess cell is blank
</commit_message>
<xml_diff>
--- a/fixtures/gstr1/demo-workbook.xlsx
+++ b/fixtures/gstr1/demo-workbook.xlsx
@@ -28,8 +28,9 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="1">
+  <numFmts count="2">
     <numFmt numFmtId="164" formatCode="yyyy-mm-dd"/>
+    <numFmt numFmtId="165" formatCode="yyyy-mm-dd h:mm:ss"/>
   </numFmts>
   <fonts count="1">
     <font>
@@ -60,9 +61,10 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -521,8 +523,10 @@
           <t>INV-001</t>
         </is>
       </c>
-      <c r="D5" s="1" t="n">
-        <v>42930</v>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>14-Jul-2017</t>
+        </is>
       </c>
       <c r="E5" t="n">
         <v>118000</v>
@@ -565,8 +569,10 @@
           <t>INV-002</t>
         </is>
       </c>
-      <c r="D6" s="1" t="n">
-        <v>42931</v>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>15-Jul-2017</t>
+        </is>
       </c>
       <c r="E6" t="n">
         <v>80000</v>
@@ -609,8 +615,10 @@
           <t>INV-002</t>
         </is>
       </c>
-      <c r="D7" s="1" t="n">
-        <v>42931</v>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>15-Jul-2017</t>
+        </is>
       </c>
       <c r="E7" t="n">
         <v>80000</v>
@@ -653,8 +661,10 @@
           <t>INV-003</t>
         </is>
       </c>
-      <c r="D8" s="1" t="n">
-        <v>42932</v>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>16-Jul-2017</t>
+        </is>
       </c>
       <c r="E8" t="n">
         <v>44800</v>
@@ -697,8 +707,10 @@
           <t>INV-004</t>
         </is>
       </c>
-      <c r="D9" s="1" t="n">
-        <v>42936</v>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>20-Jul-2017</t>
+        </is>
       </c>
       <c r="E9" t="n">
         <v>24100</v>
@@ -744,8 +756,10 @@
           <t>INV-005</t>
         </is>
       </c>
-      <c r="D10" s="1" t="n">
-        <v>42937</v>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>21-Jul-2017</t>
+        </is>
       </c>
       <c r="E10" t="n">
         <v>30000</v>
@@ -788,8 +802,10 @@
           <t>INV-006</t>
         </is>
       </c>
-      <c r="D11" s="1" t="n">
-        <v>42938</v>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>22-Jul-2017</t>
+        </is>
       </c>
       <c r="E11" t="n">
         <v>111700</v>
@@ -913,16 +929,20 @@
           <t>UN-001</t>
         </is>
       </c>
-      <c r="C5" s="1" t="n">
-        <v>42930</v>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>14-Jul-2017</t>
+        </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
           <t>UN-001-R</t>
         </is>
       </c>
-      <c r="E5" s="1" t="n">
-        <v>42983</v>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>05-Sep-2017</t>
+        </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
@@ -955,16 +975,20 @@
           <t>UN-002</t>
         </is>
       </c>
-      <c r="C6" s="1" t="n">
-        <v>42931</v>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>15-Jul-2017</t>
+        </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
           <t>UN-002</t>
         </is>
       </c>
-      <c r="E6" s="1" t="n">
-        <v>42984</v>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>06-Sep-2017</t>
+        </is>
       </c>
       <c r="F6" t="inlineStr">
         <is>
@@ -992,16 +1016,20 @@
           <t>UN-003</t>
         </is>
       </c>
-      <c r="C7" s="1" t="n">
-        <v>42932</v>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>16-Jul-2017</t>
+        </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
           <t>UN-003-R</t>
         </is>
       </c>
-      <c r="E7" s="1" t="n">
-        <v>42985</v>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>07-Sep-2017</t>
+        </is>
       </c>
       <c r="F7" t="inlineStr">
         <is>
@@ -1652,16 +1680,20 @@
           <t>INV-001</t>
         </is>
       </c>
-      <c r="D5" s="1" t="n">
-        <v>42930</v>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>14-Jul-2017</t>
+        </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
           <t>INV-001-R</t>
         </is>
       </c>
-      <c r="F5" s="1" t="n">
-        <v>42983</v>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>05-Sep-2017</t>
+        </is>
       </c>
       <c r="G5" t="n">
         <v>118000</v>
@@ -1704,16 +1736,20 @@
           <t>INV-002</t>
         </is>
       </c>
-      <c r="D6" s="1" t="n">
-        <v>42931</v>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>15-Jul-2017</t>
+        </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
           <t>INV-002</t>
         </is>
       </c>
-      <c r="F6" s="1" t="n">
-        <v>42984</v>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>06-Sep-2017</t>
+        </is>
       </c>
       <c r="G6" t="n">
         <v>80000</v>
@@ -1756,16 +1792,20 @@
           <t>INV-002</t>
         </is>
       </c>
-      <c r="D7" s="1" t="n">
-        <v>42931</v>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>15-Jul-2017</t>
+        </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
           <t>INV-002</t>
         </is>
       </c>
-      <c r="F7" s="1" t="n">
-        <v>42984</v>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>06-Sep-2017</t>
+        </is>
       </c>
       <c r="G7" t="n">
         <v>80000</v>
@@ -1808,16 +1848,20 @@
           <t>INV-003</t>
         </is>
       </c>
-      <c r="D8" s="1" t="n">
-        <v>42936</v>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>20-Jul-2017</t>
+        </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
           <t>INV-003-R</t>
         </is>
       </c>
-      <c r="F8" s="1" t="n">
-        <v>42985</v>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>07-Sep-2017</t>
+        </is>
       </c>
       <c r="G8" t="n">
         <v>24100</v>
@@ -1863,16 +1907,20 @@
           <t>INV-004</t>
         </is>
       </c>
-      <c r="D9" s="1" t="n">
-        <v>42937</v>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>21-Jul-2017</t>
+        </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
           <t>INV-004-R</t>
         </is>
       </c>
-      <c r="F9" s="1" t="n">
-        <v>42986</v>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t>08-Sep-2017</t>
+        </is>
       </c>
       <c r="G9" t="n">
         <v>111700</v>
@@ -1976,8 +2024,10 @@
           <t>INV-L001</t>
         </is>
       </c>
-      <c r="B5" s="1" t="n">
-        <v>42930</v>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>14-Jul-2017</t>
+        </is>
       </c>
       <c r="C5" t="n">
         <v>295000</v>
@@ -2000,8 +2050,10 @@
           <t>INV-L002</t>
         </is>
       </c>
-      <c r="B6" s="1" t="n">
-        <v>42931</v>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>15-Jul-2017</t>
+        </is>
       </c>
       <c r="C6" t="n">
         <v>283000</v>
@@ -2024,8 +2076,10 @@
           <t>INV-L002</t>
         </is>
       </c>
-      <c r="B7" s="1" t="n">
-        <v>42931</v>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>15-Jul-2017</t>
+        </is>
       </c>
       <c r="C7" t="n">
         <v>283000</v>
@@ -2048,8 +2102,10 @@
           <t>INV-L003</t>
         </is>
       </c>
-      <c r="B8" s="1" t="n">
-        <v>42936</v>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>20-Jul-2017</t>
+        </is>
       </c>
       <c r="C8" t="n">
         <v>278500</v>
@@ -2075,8 +2131,10 @@
           <t>INV-L004</t>
         </is>
       </c>
-      <c r="B9" s="1" t="n">
-        <v>42937</v>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>21-Jul-2017</t>
+        </is>
       </c>
       <c r="C9" t="n">
         <v>265250</v>
@@ -2180,8 +2238,10 @@
           <t>INV-L001</t>
         </is>
       </c>
-      <c r="B5" s="1" t="n">
-        <v>42930</v>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>14-Jul-2017</t>
+        </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
@@ -2193,8 +2253,10 @@
           <t>INV-L001-R</t>
         </is>
       </c>
-      <c r="E5" s="1" t="n">
-        <v>42983</v>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>05-Sep-2017</t>
+        </is>
       </c>
       <c r="F5" t="n">
         <v>295000</v>
@@ -2212,8 +2274,10 @@
           <t>INV-L002</t>
         </is>
       </c>
-      <c r="B6" s="1" t="n">
-        <v>42931</v>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>15-Jul-2017</t>
+        </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
@@ -2225,8 +2289,10 @@
           <t>INV-L002</t>
         </is>
       </c>
-      <c r="E6" s="1" t="n">
-        <v>42984</v>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>06-Sep-2017</t>
+        </is>
       </c>
       <c r="F6" t="n">
         <v>283000</v>
@@ -2244,8 +2310,10 @@
           <t>INV-L002</t>
         </is>
       </c>
-      <c r="B7" s="1" t="n">
-        <v>42931</v>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>15-Jul-2017</t>
+        </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
@@ -2257,8 +2325,10 @@
           <t>INV-L002</t>
         </is>
       </c>
-      <c r="E7" s="1" t="n">
-        <v>42984</v>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>06-Sep-2017</t>
+        </is>
       </c>
       <c r="F7" t="n">
         <v>283000</v>
@@ -2276,8 +2346,10 @@
           <t>INV-L003</t>
         </is>
       </c>
-      <c r="B8" s="1" t="n">
-        <v>42936</v>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>20-Jul-2017</t>
+        </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
@@ -2289,8 +2361,10 @@
           <t>INV-L003-R</t>
         </is>
       </c>
-      <c r="E8" s="1" t="n">
-        <v>42985</v>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>07-Sep-2017</t>
+        </is>
       </c>
       <c r="F8" t="n">
         <v>278500</v>
@@ -2311,8 +2385,10 @@
           <t>INV-L004</t>
         </is>
       </c>
-      <c r="B9" s="1" t="n">
-        <v>42937</v>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>21-Jul-2017</t>
+        </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
@@ -2324,8 +2400,10 @@
           <t>INV-L004-R</t>
         </is>
       </c>
-      <c r="E9" s="1" t="n">
-        <v>42986</v>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>08-Sep-2017</t>
+        </is>
       </c>
       <c r="F9" t="n">
         <v>265250</v>
@@ -2812,8 +2890,10 @@
           <t>CN-001</t>
         </is>
       </c>
-      <c r="D5" s="1" t="n">
-        <v>42930</v>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>14-Jul-2017</t>
+        </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
@@ -2861,8 +2941,10 @@
           <t>CN-002</t>
         </is>
       </c>
-      <c r="D6" s="1" t="n">
-        <v>42931</v>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>15-Jul-2017</t>
+        </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
@@ -2910,8 +2992,10 @@
           <t>CN-003</t>
         </is>
       </c>
-      <c r="D7" s="1" t="n">
-        <v>42936</v>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>20-Jul-2017</t>
+        </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
@@ -2962,8 +3046,10 @@
           <t>CN-003</t>
         </is>
       </c>
-      <c r="D8" s="1" t="n">
-        <v>42936</v>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>20-Jul-2017</t>
+        </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
@@ -3109,16 +3195,20 @@
           <t>CN-001</t>
         </is>
       </c>
-      <c r="D5" s="1" t="n">
-        <v>42930</v>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>14-Jul-2017</t>
+        </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
           <t>CN-001-R</t>
         </is>
       </c>
-      <c r="F5" s="1" t="n">
-        <v>42983</v>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>05-Sep-2017</t>
+        </is>
       </c>
       <c r="G5" t="inlineStr">
         <is>
@@ -3166,16 +3256,20 @@
           <t>CN-002</t>
         </is>
       </c>
-      <c r="D6" s="1" t="n">
-        <v>42931</v>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>15-Jul-2017</t>
+        </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
           <t>CN-002</t>
         </is>
       </c>
-      <c r="F6" s="1" t="n">
-        <v>42984</v>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>06-Sep-2017</t>
+        </is>
       </c>
       <c r="G6" t="inlineStr">
         <is>
@@ -3223,16 +3317,20 @@
           <t>CN-003</t>
         </is>
       </c>
-      <c r="D7" s="1" t="n">
-        <v>42936</v>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>20-Jul-2017</t>
+        </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
           <t>CN-003-R</t>
         </is>
       </c>
-      <c r="F7" s="1" t="n">
-        <v>42985</v>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>07-Sep-2017</t>
+        </is>
       </c>
       <c r="G7" t="inlineStr">
         <is>
@@ -3354,8 +3452,10 @@
           <t>UN-001</t>
         </is>
       </c>
-      <c r="C5" s="1" t="n">
-        <v>42930</v>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>14-Jul-2017</t>
+        </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
@@ -3388,8 +3488,10 @@
           <t>UN-001</t>
         </is>
       </c>
-      <c r="C6" s="1" t="n">
-        <v>42930</v>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>14-Jul-2017</t>
+        </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
@@ -3425,8 +3527,10 @@
           <t>UN-002</t>
         </is>
       </c>
-      <c r="C7" s="1" t="n">
-        <v>42931</v>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>15-Jul-2017</t>
+        </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
@@ -3454,8 +3558,10 @@
           <t>UN-003</t>
         </is>
       </c>
-      <c r="C8" s="1" t="n">
-        <v>42932</v>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>16-Jul-2017</t>
+        </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
feat(gstr1): exports and amended exports (exp, expa)
</commit_message>
<xml_diff>
--- a/fixtures/gstr1/demo-workbook.xlsx
+++ b/fixtures/gstr1/demo-workbook.xlsx
@@ -17,9 +17,11 @@
     <sheet name="cdnra" sheetId="8" state="visible" r:id="rId8"/>
     <sheet name="cdnur" sheetId="9" state="visible" r:id="rId9"/>
     <sheet name="cdnura" sheetId="10" state="visible" r:id="rId10"/>
-    <sheet name="docs" sheetId="11" state="visible" r:id="rId11"/>
-    <sheet name="hsn(b2b)" sheetId="12" state="visible" r:id="rId12"/>
-    <sheet name="hsn(b2c)" sheetId="13" state="visible" r:id="rId13"/>
+    <sheet name="exp" sheetId="11" state="visible" r:id="rId11"/>
+    <sheet name="expa" sheetId="12" state="visible" r:id="rId12"/>
+    <sheet name="docs" sheetId="13" state="visible" r:id="rId13"/>
+    <sheet name="hsn(b2b)" sheetId="14" state="visible" r:id="rId14"/>
+    <sheet name="hsn(b2c)" sheetId="15" state="visible" r:id="rId15"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -1060,156 +1062,221 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E9"/>
+  <dimension ref="A1:J8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="inlineStr">
         <is>
-          <t>Summary for doc_issue</t>
+          <t>Summary for exp</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Nature of Document</t>
+          <t>Export Type</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Sr. No. From</t>
+          <t>Invoice Number</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>Sr. No. To</t>
+          <t>Invoice date</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>Total Number</t>
+          <t>Invoice Value</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>Cancelled</t>
+          <t>Port Code</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>Shipping Bill Number</t>
+        </is>
+      </c>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>Shipping Bill Date</t>
+        </is>
+      </c>
+      <c r="H4" t="inlineStr">
+        <is>
+          <t>Rate</t>
+        </is>
+      </c>
+      <c r="I4" t="inlineStr">
+        <is>
+          <t>Taxable Value</t>
+        </is>
+      </c>
+      <c r="J4" t="inlineStr">
+        <is>
+          <t>Cess Amount</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Invoices for outward supply</t>
+          <t>WPAY</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>INV-001</t>
+          <t>EXP-001</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>INV-100</t>
+          <t>14-Jul-2017</t>
         </is>
       </c>
       <c r="D5" t="n">
-        <v>100</v>
-      </c>
-      <c r="E5" t="n">
-        <v>2</v>
+        <v>295000</v>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>INMAA1</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>7896542</t>
+        </is>
+      </c>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>18-Jul-2017</t>
+        </is>
+      </c>
+      <c r="H5" t="n">
+        <v>18</v>
+      </c>
+      <c r="I5" t="n">
+        <v>250000</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Invoices for outward supply</t>
+          <t>WPAY</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>INV-201</t>
+          <t>EXP-001</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>INV-250</t>
+          <t>14-Jul-2017</t>
         </is>
       </c>
       <c r="D6" t="n">
-        <v>50</v>
-      </c>
-      <c r="E6" t="n">
-        <v>0</v>
+        <v>295000</v>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>INMAA1</t>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>7896542</t>
+        </is>
+      </c>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t>18-Jul-2017</t>
+        </is>
+      </c>
+      <c r="H6" t="n">
+        <v>5</v>
+      </c>
+      <c r="I6" t="n">
+        <v>20000</v>
+      </c>
+      <c r="J6" t="n">
+        <v>500</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>Credit Note</t>
+          <t>WPAY</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>CN-001</t>
+          <t>EXP-002</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>CN-010</t>
+          <t>22-Jul-2017</t>
         </is>
       </c>
       <c r="D7" t="n">
-        <v>10</v>
-      </c>
-      <c r="E7" t="n">
-        <v>1</v>
+        <v>60000</v>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>INNSA1</t>
+        </is>
+      </c>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>1234567</t>
+        </is>
+      </c>
+      <c r="G7" t="inlineStr">
+        <is>
+          <t>25-Jul-2017</t>
+        </is>
+      </c>
+      <c r="H7" t="n">
+        <v>12</v>
+      </c>
+      <c r="I7" t="n">
+        <v>50000</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>Debit Note</t>
+          <t>WOPAY</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>DN-001</t>
+          <t>EXP-003</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>DN-005</t>
+          <t>20-Jul-2017</t>
         </is>
       </c>
       <c r="D8" t="n">
-        <v>5</v>
-      </c>
-      <c r="E8" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" t="inlineStr">
-        <is>
-          <t>Delivery Challan for job work</t>
-        </is>
-      </c>
-      <c r="B9" t="inlineStr">
-        <is>
-          <t>DC-001</t>
-        </is>
-      </c>
-      <c r="C9" t="inlineStr">
-        <is>
-          <t>DC-020</t>
-        </is>
-      </c>
-      <c r="D9" t="n">
-        <v>20</v>
-      </c>
-      <c r="E9" t="n">
-        <v>3</v>
+        <v>180000</v>
+      </c>
+      <c r="H8" t="n">
+        <v>18</v>
+      </c>
+      <c r="I8" t="n">
+        <v>180000</v>
+      </c>
+      <c r="J8" t="n">
+        <v>750</v>
       </c>
     </row>
   </sheetData>
@@ -1223,68 +1290,73 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K7"/>
+  <dimension ref="A1:L6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="inlineStr">
         <is>
-          <t>Summary for hsn(b2b)</t>
+          <t>Summary for expa</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>HSN</t>
+          <t>Export Type</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Description</t>
+          <t>Original Invoice Number</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>UQC</t>
+          <t>Original Invoice date</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>Total Quantity</t>
+          <t>Revised Invoice Number</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>Total Value</t>
+          <t>Revised Invoice date</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
+          <t>Invoice Value</t>
+        </is>
+      </c>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>Port Code</t>
+        </is>
+      </c>
+      <c r="H4" t="inlineStr">
+        <is>
+          <t>Shipping Bill Number</t>
+        </is>
+      </c>
+      <c r="I4" t="inlineStr">
+        <is>
+          <t>Shipping Bill Date</t>
+        </is>
+      </c>
+      <c r="J4" t="inlineStr">
+        <is>
           <t>Rate</t>
         </is>
       </c>
-      <c r="G4" t="inlineStr">
+      <c r="K4" t="inlineStr">
         <is>
           <t>Taxable Value</t>
         </is>
       </c>
-      <c r="H4" t="inlineStr">
-        <is>
-          <t>Integrated Tax Amount</t>
-        </is>
-      </c>
-      <c r="I4" t="inlineStr">
-        <is>
-          <t>Central Tax Amount</t>
-        </is>
-      </c>
-      <c r="J4" t="inlineStr">
-        <is>
-          <t>State/UT Tax Amount</t>
-        </is>
-      </c>
-      <c r="K4" t="inlineStr">
+      <c r="L4" t="inlineStr">
         <is>
           <t>Cess Amount</t>
         </is>
@@ -1293,100 +1365,96 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>0101</t>
+          <t>WPAY</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Live horses</t>
+          <t>EXP-A01</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>NOS-NUMBERS</t>
-        </is>
-      </c>
-      <c r="D5" t="n">
-        <v>10</v>
-      </c>
-      <c r="E5" t="n">
-        <v>118000</v>
+          <t>14-Jul-2017</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>EXP-A01-R</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>20-Jul-2017</t>
+        </is>
       </c>
       <c r="F5" t="n">
+        <v>295000</v>
+      </c>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>INMAA1</t>
+        </is>
+      </c>
+      <c r="H5" t="inlineStr">
+        <is>
+          <t>7896542</t>
+        </is>
+      </c>
+      <c r="I5" t="inlineStr">
+        <is>
+          <t>22-Jul-2017</t>
+        </is>
+      </c>
+      <c r="J5" t="n">
         <v>18</v>
       </c>
-      <c r="G5" t="n">
-        <v>100000</v>
-      </c>
-      <c r="H5" t="n">
-        <v>18000</v>
+      <c r="K5" t="n">
+        <v>250000</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>0102</t>
+          <t>WOPAY</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Live bovine animals</t>
+          <t>EXP-A02</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>NOS-NUMBERS</t>
-        </is>
-      </c>
-      <c r="D6" t="n">
-        <v>5</v>
-      </c>
-      <c r="E6" t="n">
-        <v>52500</v>
+          <t>15-Jul-2017</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>EXP-A02</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>21-Jul-2017</t>
+        </is>
       </c>
       <c r="F6" t="n">
-        <v>5</v>
-      </c>
-      <c r="G6" t="n">
-        <v>50000</v>
-      </c>
-      <c r="H6" t="n">
-        <v>2500</v>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" t="inlineStr">
-        <is>
-          <t>1006</t>
-        </is>
-      </c>
-      <c r="B7" t="inlineStr">
-        <is>
-          <t>Rice</t>
-        </is>
-      </c>
-      <c r="C7" t="inlineStr">
-        <is>
-          <t>KGS-KILOGRAMS</t>
-        </is>
-      </c>
-      <c r="D7" t="n">
-        <v>1000</v>
-      </c>
-      <c r="E7" t="n">
-        <v>105000</v>
-      </c>
-      <c r="F7" t="n">
-        <v>5</v>
-      </c>
-      <c r="G7" t="n">
-        <v>100000</v>
-      </c>
-      <c r="I7" t="n">
-        <v>2500</v>
-      </c>
-      <c r="J7" t="n">
-        <v>2500</v>
+        <v>180000</v>
+      </c>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t>INNSA1</t>
+        </is>
+      </c>
+      <c r="J6" t="n">
+        <v>18</v>
+      </c>
+      <c r="K6" t="n">
+        <v>180000</v>
+      </c>
+      <c r="L6" t="n">
+        <v>750</v>
       </c>
     </row>
   </sheetData>
@@ -1395,6 +1463,346 @@
 </file>
 
 <file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:E9"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>Summary for doc_issue</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>Nature of Document</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>Sr. No. From</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>Sr. No. To</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>Total Number</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>Cancelled</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>Invoices for outward supply</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>INV-001</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>INV-100</t>
+        </is>
+      </c>
+      <c r="D5" t="n">
+        <v>100</v>
+      </c>
+      <c r="E5" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>Invoices for outward supply</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>INV-201</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>INV-250</t>
+        </is>
+      </c>
+      <c r="D6" t="n">
+        <v>50</v>
+      </c>
+      <c r="E6" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>Credit Note</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>CN-001</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>CN-010</t>
+        </is>
+      </c>
+      <c r="D7" t="n">
+        <v>10</v>
+      </c>
+      <c r="E7" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>Debit Note</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>DN-001</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>DN-005</t>
+        </is>
+      </c>
+      <c r="D8" t="n">
+        <v>5</v>
+      </c>
+      <c r="E8" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>Delivery Challan for job work</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>DC-001</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>DC-020</t>
+        </is>
+      </c>
+      <c r="D9" t="n">
+        <v>20</v>
+      </c>
+      <c r="E9" t="n">
+        <v>3</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:K7"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>Summary for hsn(b2b)</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>HSN</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>Description</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>UQC</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>Total Quantity</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>Total Value</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>Rate</t>
+        </is>
+      </c>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>Taxable Value</t>
+        </is>
+      </c>
+      <c r="H4" t="inlineStr">
+        <is>
+          <t>Integrated Tax Amount</t>
+        </is>
+      </c>
+      <c r="I4" t="inlineStr">
+        <is>
+          <t>Central Tax Amount</t>
+        </is>
+      </c>
+      <c r="J4" t="inlineStr">
+        <is>
+          <t>State/UT Tax Amount</t>
+        </is>
+      </c>
+      <c r="K4" t="inlineStr">
+        <is>
+          <t>Cess Amount</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>0101</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>Live horses</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>NOS-NUMBERS</t>
+        </is>
+      </c>
+      <c r="D5" t="n">
+        <v>10</v>
+      </c>
+      <c r="E5" t="n">
+        <v>118000</v>
+      </c>
+      <c r="F5" t="n">
+        <v>18</v>
+      </c>
+      <c r="G5" t="n">
+        <v>100000</v>
+      </c>
+      <c r="H5" t="n">
+        <v>18000</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>0102</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>Live bovine animals</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>NOS-NUMBERS</t>
+        </is>
+      </c>
+      <c r="D6" t="n">
+        <v>5</v>
+      </c>
+      <c r="E6" t="n">
+        <v>52500</v>
+      </c>
+      <c r="F6" t="n">
+        <v>5</v>
+      </c>
+      <c r="G6" t="n">
+        <v>50000</v>
+      </c>
+      <c r="H6" t="n">
+        <v>2500</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>1006</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>Rice</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>KGS-KILOGRAMS</t>
+        </is>
+      </c>
+      <c r="D7" t="n">
+        <v>1000</v>
+      </c>
+      <c r="E7" t="n">
+        <v>105000</v>
+      </c>
+      <c r="F7" t="n">
+        <v>5</v>
+      </c>
+      <c r="G7" t="n">
+        <v>100000</v>
+      </c>
+      <c r="I7" t="n">
+        <v>2500</v>
+      </c>
+      <c r="J7" t="n">
+        <v>2500</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet15.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>

</xml_diff>

<commit_message>
feat(gstr1): nil rated, exempted and non-GST supplies (exemp)
</commit_message>
<xml_diff>
--- a/fixtures/gstr1/demo-workbook.xlsx
+++ b/fixtures/gstr1/demo-workbook.xlsx
@@ -19,9 +19,10 @@
     <sheet name="cdnura" sheetId="10" state="visible" r:id="rId10"/>
     <sheet name="exp" sheetId="11" state="visible" r:id="rId11"/>
     <sheet name="expa" sheetId="12" state="visible" r:id="rId12"/>
-    <sheet name="docs" sheetId="13" state="visible" r:id="rId13"/>
-    <sheet name="hsn(b2b)" sheetId="14" state="visible" r:id="rId14"/>
-    <sheet name="hsn(b2c)" sheetId="15" state="visible" r:id="rId15"/>
+    <sheet name="exemp" sheetId="13" state="visible" r:id="rId13"/>
+    <sheet name="docs" sheetId="14" state="visible" r:id="rId14"/>
+    <sheet name="hsn(b2b)" sheetId="15" state="visible" r:id="rId15"/>
+    <sheet name="hsn(b2c)" sheetId="16" state="visible" r:id="rId16"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -1468,156 +1469,97 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E9"/>
+  <dimension ref="A1:D8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="inlineStr">
         <is>
-          <t>Summary for doc_issue</t>
+          <t>Summary For Nil rated, exempted and non GST outward supplies (8)</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Nature of Document</t>
+          <t>Description</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Sr. No. From</t>
+          <t>Nil Rated Supplies</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>Sr. No. To</t>
+          <t>Exempted(other than nil rated/non GST supply)</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>Total Number</t>
-        </is>
-      </c>
-      <c r="E4" t="inlineStr">
-        <is>
-          <t>Cancelled</t>
+          <t>Non-GST Supplies</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Invoices for outward supply</t>
-        </is>
-      </c>
-      <c r="B5" t="inlineStr">
-        <is>
-          <t>INV-001</t>
-        </is>
-      </c>
-      <c r="C5" t="inlineStr">
-        <is>
-          <t>INV-100</t>
-        </is>
+          <t>Inter-State supplies to registered persons</t>
+        </is>
+      </c>
+      <c r="B5" t="n">
+        <v>21143</v>
+      </c>
+      <c r="C5" t="n">
+        <v>51235</v>
       </c>
       <c r="D5" t="n">
-        <v>100</v>
-      </c>
-      <c r="E5" t="n">
-        <v>2</v>
+        <v>5213</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Invoices for outward supply</t>
-        </is>
-      </c>
-      <c r="B6" t="inlineStr">
-        <is>
-          <t>INV-201</t>
-        </is>
-      </c>
-      <c r="C6" t="inlineStr">
-        <is>
-          <t>INV-250</t>
-        </is>
+          <t>Intra-State supplies to registered persons</t>
+        </is>
+      </c>
+      <c r="B6" t="n">
+        <v>525</v>
+      </c>
+      <c r="C6" t="n">
+        <v>52135</v>
       </c>
       <c r="D6" t="n">
-        <v>50</v>
-      </c>
-      <c r="E6" t="n">
-        <v>0</v>
+        <v>5435</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>Credit Note</t>
-        </is>
-      </c>
-      <c r="B7" t="inlineStr">
-        <is>
-          <t>CN-001</t>
-        </is>
-      </c>
-      <c r="C7" t="inlineStr">
-        <is>
-          <t>CN-010</t>
-        </is>
+          <t>Inter-State supplies to unregistered persons</t>
+        </is>
+      </c>
+      <c r="B7" t="n">
+        <v>1234</v>
+      </c>
+      <c r="C7" t="n">
+        <v>512</v>
       </c>
       <c r="D7" t="n">
-        <v>10</v>
-      </c>
-      <c r="E7" t="n">
-        <v>1</v>
+        <v>5123</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>Debit Note</t>
-        </is>
-      </c>
-      <c r="B8" t="inlineStr">
-        <is>
-          <t>DN-001</t>
-        </is>
-      </c>
-      <c r="C8" t="inlineStr">
-        <is>
-          <t>DN-005</t>
-        </is>
-      </c>
-      <c r="D8" t="n">
-        <v>5</v>
-      </c>
-      <c r="E8" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" t="inlineStr">
-        <is>
-          <t>Delivery Challan for job work</t>
-        </is>
-      </c>
-      <c r="B9" t="inlineStr">
-        <is>
-          <t>DC-001</t>
-        </is>
-      </c>
-      <c r="C9" t="inlineStr">
-        <is>
-          <t>DC-020</t>
-        </is>
-      </c>
-      <c r="D9" t="n">
-        <v>20</v>
-      </c>
-      <c r="E9" t="n">
-        <v>3</v>
+          <t>Intra-State supplies to unregistered persons</t>
+        </is>
+      </c>
+      <c r="B8" t="n">
+        <v>684</v>
+      </c>
+      <c r="C8" t="n">
+        <v>998</v>
       </c>
     </row>
   </sheetData>
@@ -1631,170 +1573,156 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K7"/>
+  <dimension ref="A1:E9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="inlineStr">
         <is>
-          <t>Summary for hsn(b2b)</t>
+          <t>Summary for doc_issue</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>HSN</t>
+          <t>Nature of Document</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Description</t>
+          <t>Sr. No. From</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>UQC</t>
+          <t>Sr. No. To</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>Total Quantity</t>
+          <t>Total Number</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>Total Value</t>
-        </is>
-      </c>
-      <c r="F4" t="inlineStr">
-        <is>
-          <t>Rate</t>
-        </is>
-      </c>
-      <c r="G4" t="inlineStr">
-        <is>
-          <t>Taxable Value</t>
-        </is>
-      </c>
-      <c r="H4" t="inlineStr">
-        <is>
-          <t>Integrated Tax Amount</t>
-        </is>
-      </c>
-      <c r="I4" t="inlineStr">
-        <is>
-          <t>Central Tax Amount</t>
-        </is>
-      </c>
-      <c r="J4" t="inlineStr">
-        <is>
-          <t>State/UT Tax Amount</t>
-        </is>
-      </c>
-      <c r="K4" t="inlineStr">
-        <is>
-          <t>Cess Amount</t>
+          <t>Cancelled</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>0101</t>
+          <t>Invoices for outward supply</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Live horses</t>
+          <t>INV-001</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>NOS-NUMBERS</t>
+          <t>INV-100</t>
         </is>
       </c>
       <c r="D5" t="n">
-        <v>10</v>
+        <v>100</v>
       </c>
       <c r="E5" t="n">
-        <v>118000</v>
-      </c>
-      <c r="F5" t="n">
-        <v>18</v>
-      </c>
-      <c r="G5" t="n">
-        <v>100000</v>
-      </c>
-      <c r="H5" t="n">
-        <v>18000</v>
+        <v>2</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>0102</t>
+          <t>Invoices for outward supply</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Live bovine animals</t>
+          <t>INV-201</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>NOS-NUMBERS</t>
+          <t>INV-250</t>
         </is>
       </c>
       <c r="D6" t="n">
-        <v>5</v>
+        <v>50</v>
       </c>
       <c r="E6" t="n">
-        <v>52500</v>
-      </c>
-      <c r="F6" t="n">
-        <v>5</v>
-      </c>
-      <c r="G6" t="n">
-        <v>50000</v>
-      </c>
-      <c r="H6" t="n">
-        <v>2500</v>
+        <v>0</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>1006</t>
+          <t>Credit Note</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>Rice</t>
+          <t>CN-001</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>KGS-KILOGRAMS</t>
+          <t>CN-010</t>
         </is>
       </c>
       <c r="D7" t="n">
-        <v>1000</v>
+        <v>10</v>
       </c>
       <c r="E7" t="n">
-        <v>105000</v>
-      </c>
-      <c r="F7" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>Debit Note</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>DN-001</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>DN-005</t>
+        </is>
+      </c>
+      <c r="D8" t="n">
         <v>5</v>
       </c>
-      <c r="G7" t="n">
-        <v>100000</v>
-      </c>
-      <c r="I7" t="n">
-        <v>2500</v>
-      </c>
-      <c r="J7" t="n">
-        <v>2500</v>
+      <c r="E8" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>Delivery Challan for job work</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>DC-001</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>DC-020</t>
+        </is>
+      </c>
+      <c r="D9" t="n">
+        <v>20</v>
+      </c>
+      <c r="E9" t="n">
+        <v>3</v>
       </c>
     </row>
   </sheetData>
@@ -1814,6 +1742,183 @@
     <row r="1">
       <c r="A1" t="inlineStr">
         <is>
+          <t>Summary for hsn(b2b)</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>HSN</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>Description</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>UQC</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>Total Quantity</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>Total Value</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>Rate</t>
+        </is>
+      </c>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>Taxable Value</t>
+        </is>
+      </c>
+      <c r="H4" t="inlineStr">
+        <is>
+          <t>Integrated Tax Amount</t>
+        </is>
+      </c>
+      <c r="I4" t="inlineStr">
+        <is>
+          <t>Central Tax Amount</t>
+        </is>
+      </c>
+      <c r="J4" t="inlineStr">
+        <is>
+          <t>State/UT Tax Amount</t>
+        </is>
+      </c>
+      <c r="K4" t="inlineStr">
+        <is>
+          <t>Cess Amount</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>0101</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>Live horses</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>NOS-NUMBERS</t>
+        </is>
+      </c>
+      <c r="D5" t="n">
+        <v>10</v>
+      </c>
+      <c r="E5" t="n">
+        <v>118000</v>
+      </c>
+      <c r="F5" t="n">
+        <v>18</v>
+      </c>
+      <c r="G5" t="n">
+        <v>100000</v>
+      </c>
+      <c r="H5" t="n">
+        <v>18000</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>0102</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>Live bovine animals</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>NOS-NUMBERS</t>
+        </is>
+      </c>
+      <c r="D6" t="n">
+        <v>5</v>
+      </c>
+      <c r="E6" t="n">
+        <v>52500</v>
+      </c>
+      <c r="F6" t="n">
+        <v>5</v>
+      </c>
+      <c r="G6" t="n">
+        <v>50000</v>
+      </c>
+      <c r="H6" t="n">
+        <v>2500</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>1006</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>Rice</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>KGS-KILOGRAMS</t>
+        </is>
+      </c>
+      <c r="D7" t="n">
+        <v>1000</v>
+      </c>
+      <c r="E7" t="n">
+        <v>105000</v>
+      </c>
+      <c r="F7" t="n">
+        <v>5</v>
+      </c>
+      <c r="G7" t="n">
+        <v>100000</v>
+      </c>
+      <c r="I7" t="n">
+        <v>2500</v>
+      </c>
+      <c r="J7" t="n">
+        <v>2500</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet16.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:K7"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
           <t>Summary for hsn(b2c)</t>
         </is>
       </c>

</xml_diff>

<commit_message>
feat(gstr1): advances received and adjusted (at, ata, atadj, atadja)
</commit_message>
<xml_diff>
--- a/fixtures/gstr1/demo-workbook.xlsx
+++ b/fixtures/gstr1/demo-workbook.xlsx
@@ -19,10 +19,14 @@
     <sheet name="cdnura" sheetId="10" state="visible" r:id="rId10"/>
     <sheet name="exp" sheetId="11" state="visible" r:id="rId11"/>
     <sheet name="expa" sheetId="12" state="visible" r:id="rId12"/>
-    <sheet name="exemp" sheetId="13" state="visible" r:id="rId13"/>
-    <sheet name="docs" sheetId="14" state="visible" r:id="rId14"/>
-    <sheet name="hsn(b2b)" sheetId="15" state="visible" r:id="rId15"/>
-    <sheet name="hsn(b2c)" sheetId="16" state="visible" r:id="rId16"/>
+    <sheet name="at" sheetId="13" state="visible" r:id="rId13"/>
+    <sheet name="ata" sheetId="14" state="visible" r:id="rId14"/>
+    <sheet name="atadj" sheetId="15" state="visible" r:id="rId15"/>
+    <sheet name="atadja" sheetId="16" state="visible" r:id="rId16"/>
+    <sheet name="exemp" sheetId="17" state="visible" r:id="rId17"/>
+    <sheet name="docs" sheetId="18" state="visible" r:id="rId18"/>
+    <sheet name="hsn(b2b)" sheetId="19" state="visible" r:id="rId19"/>
+    <sheet name="hsn(b2c)" sheetId="20" state="visible" r:id="rId20"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -1469,97 +1473,83 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D8"/>
+  <dimension ref="A1:E7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="inlineStr">
         <is>
-          <t>Summary For Nil rated, exempted and non GST outward supplies (8)</t>
+          <t>Summary for at</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Description</t>
+          <t>Place Of Supply</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Nil Rated Supplies</t>
+          <t>Applicable % of Tax Rate</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>Exempted(other than nil rated/non GST supply)</t>
+          <t>Rate</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>Non-GST Supplies</t>
+          <t>Gross Advance Received</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>Cess Amount</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Inter-State supplies to registered persons</t>
-        </is>
-      </c>
-      <c r="B5" t="n">
-        <v>21143</v>
+          <t>37-Andhra Pradesh</t>
+        </is>
       </c>
       <c r="C5" t="n">
-        <v>51235</v>
+        <v>18</v>
       </c>
       <c r="D5" t="n">
-        <v>5213</v>
+        <v>100000</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Intra-State supplies to registered persons</t>
-        </is>
-      </c>
-      <c r="B6" t="n">
-        <v>525</v>
+          <t>37-Andhra Pradesh</t>
+        </is>
       </c>
       <c r="C6" t="n">
-        <v>52135</v>
+        <v>5</v>
       </c>
       <c r="D6" t="n">
-        <v>5435</v>
+        <v>50000</v>
+      </c>
+      <c r="E6" t="n">
+        <v>1500</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>Inter-State supplies to unregistered persons</t>
-        </is>
-      </c>
-      <c r="B7" t="n">
-        <v>1234</v>
+          <t>27-Maharashtra</t>
+        </is>
       </c>
       <c r="C7" t="n">
-        <v>512</v>
+        <v>12</v>
       </c>
       <c r="D7" t="n">
-        <v>5123</v>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" t="inlineStr">
-        <is>
-          <t>Intra-State supplies to unregistered persons</t>
-        </is>
-      </c>
-      <c r="B8" t="n">
-        <v>684</v>
-      </c>
-      <c r="C8" t="n">
-        <v>998</v>
+        <v>80000</v>
       </c>
     </row>
   </sheetData>
@@ -1573,156 +1563,100 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E9"/>
+  <dimension ref="A1:G6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="inlineStr">
         <is>
-          <t>Summary for doc_issue</t>
+          <t>Summary for ata</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Nature of Document</t>
+          <t>Financial Year</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Sr. No. From</t>
+          <t>Original Month</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>Sr. No. To</t>
+          <t>Original Place Of Supply</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>Total Number</t>
+          <t>Applicable % of Tax Rate</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>Cancelled</t>
+          <t>Rate</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>Gross Advance Received</t>
+        </is>
+      </c>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>Cess Amount</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Invoices for outward supply</t>
+          <t>2017-18</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>INV-001</t>
+          <t>JULY</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>INV-100</t>
-        </is>
-      </c>
-      <c r="D5" t="n">
-        <v>100</v>
+          <t>37-Andhra Pradesh</t>
+        </is>
       </c>
       <c r="E5" t="n">
-        <v>2</v>
+        <v>18</v>
+      </c>
+      <c r="F5" t="n">
+        <v>100000</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Invoices for outward supply</t>
+          <t>2017-18</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>INV-201</t>
+          <t>JULY</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>INV-250</t>
-        </is>
-      </c>
-      <c r="D6" t="n">
-        <v>50</v>
+          <t>27-Maharashtra</t>
+        </is>
       </c>
       <c r="E6" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" t="inlineStr">
-        <is>
-          <t>Credit Note</t>
-        </is>
-      </c>
-      <c r="B7" t="inlineStr">
-        <is>
-          <t>CN-001</t>
-        </is>
-      </c>
-      <c r="C7" t="inlineStr">
-        <is>
-          <t>CN-010</t>
-        </is>
-      </c>
-      <c r="D7" t="n">
-        <v>10</v>
-      </c>
-      <c r="E7" t="n">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" t="inlineStr">
-        <is>
-          <t>Debit Note</t>
-        </is>
-      </c>
-      <c r="B8" t="inlineStr">
-        <is>
-          <t>DN-001</t>
-        </is>
-      </c>
-      <c r="C8" t="inlineStr">
-        <is>
-          <t>DN-005</t>
-        </is>
-      </c>
-      <c r="D8" t="n">
-        <v>5</v>
-      </c>
-      <c r="E8" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" t="inlineStr">
-        <is>
-          <t>Delivery Challan for job work</t>
-        </is>
-      </c>
-      <c r="B9" t="inlineStr">
-        <is>
-          <t>DC-001</t>
-        </is>
-      </c>
-      <c r="C9" t="inlineStr">
-        <is>
-          <t>DC-020</t>
-        </is>
-      </c>
-      <c r="D9" t="n">
-        <v>20</v>
-      </c>
-      <c r="E9" t="n">
-        <v>3</v>
+        <v>12</v>
+      </c>
+      <c r="F6" t="n">
+        <v>80000</v>
+      </c>
+      <c r="G6" t="n">
+        <v>500</v>
       </c>
     </row>
   </sheetData>
@@ -1736,68 +1670,38 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K7"/>
+  <dimension ref="A1:E6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="inlineStr">
         <is>
-          <t>Summary for hsn(b2b)</t>
+          <t>Summary for atadj</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>HSN</t>
+          <t>Place Of Supply</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Description</t>
+          <t>Applicable % of Tax Rate</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>UQC</t>
+          <t>Rate</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>Total Quantity</t>
+          <t>Gross Advance Adjusted</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
-        <is>
-          <t>Total Value</t>
-        </is>
-      </c>
-      <c r="F4" t="inlineStr">
-        <is>
-          <t>Rate</t>
-        </is>
-      </c>
-      <c r="G4" t="inlineStr">
-        <is>
-          <t>Taxable Value</t>
-        </is>
-      </c>
-      <c r="H4" t="inlineStr">
-        <is>
-          <t>Integrated Tax Amount</t>
-        </is>
-      </c>
-      <c r="I4" t="inlineStr">
-        <is>
-          <t>Central Tax Amount</t>
-        </is>
-      </c>
-      <c r="J4" t="inlineStr">
-        <is>
-          <t>State/UT Tax Amount</t>
-        </is>
-      </c>
-      <c r="K4" t="inlineStr">
         <is>
           <t>Cess Amount</t>
         </is>
@@ -1806,100 +1710,30 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>0101</t>
-        </is>
-      </c>
-      <c r="B5" t="inlineStr">
-        <is>
-          <t>Live horses</t>
-        </is>
-      </c>
-      <c r="C5" t="inlineStr">
-        <is>
-          <t>NOS-NUMBERS</t>
-        </is>
+          <t>37-Andhra Pradesh</t>
+        </is>
+      </c>
+      <c r="C5" t="n">
+        <v>18</v>
       </c>
       <c r="D5" t="n">
-        <v>10</v>
+        <v>30000</v>
       </c>
       <c r="E5" t="n">
-        <v>118000</v>
-      </c>
-      <c r="F5" t="n">
-        <v>18</v>
-      </c>
-      <c r="G5" t="n">
-        <v>100000</v>
-      </c>
-      <c r="H5" t="n">
-        <v>18000</v>
+        <v>2300</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>0102</t>
-        </is>
-      </c>
-      <c r="B6" t="inlineStr">
-        <is>
-          <t>Live bovine animals</t>
-        </is>
-      </c>
-      <c r="C6" t="inlineStr">
-        <is>
-          <t>NOS-NUMBERS</t>
-        </is>
+          <t>27-Maharashtra</t>
+        </is>
+      </c>
+      <c r="C6" t="n">
+        <v>12</v>
       </c>
       <c r="D6" t="n">
-        <v>5</v>
-      </c>
-      <c r="E6" t="n">
-        <v>52500</v>
-      </c>
-      <c r="F6" t="n">
-        <v>5</v>
-      </c>
-      <c r="G6" t="n">
-        <v>50000</v>
-      </c>
-      <c r="H6" t="n">
-        <v>2500</v>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" t="inlineStr">
-        <is>
-          <t>1006</t>
-        </is>
-      </c>
-      <c r="B7" t="inlineStr">
-        <is>
-          <t>Rice</t>
-        </is>
-      </c>
-      <c r="C7" t="inlineStr">
-        <is>
-          <t>KGS-KILOGRAMS</t>
-        </is>
-      </c>
-      <c r="D7" t="n">
-        <v>1000</v>
-      </c>
-      <c r="E7" t="n">
-        <v>105000</v>
-      </c>
-      <c r="F7" t="n">
-        <v>5</v>
-      </c>
-      <c r="G7" t="n">
-        <v>100000</v>
-      </c>
-      <c r="I7" t="n">
-        <v>2500</v>
-      </c>
-      <c r="J7" t="n">
-        <v>2500</v>
+        <v>20000</v>
       </c>
     </row>
   </sheetData>
@@ -1913,13 +1747,364 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
+  <dimension ref="A1:G5"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>Summary for atadja</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>Financial Year</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>Original Month</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>Original Place Of Supply</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>Applicable % of Tax Rate</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>Rate</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>Gross Advance Adjusted</t>
+        </is>
+      </c>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>Cess Amount</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>2017-18</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>JULY</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>37-Andhra Pradesh</t>
+        </is>
+      </c>
+      <c r="E5" t="n">
+        <v>18</v>
+      </c>
+      <c r="F5" t="n">
+        <v>30000</v>
+      </c>
+      <c r="G5" t="n">
+        <v>2300</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet17.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:D8"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>Summary For Nil rated, exempted and non GST outward supplies (8)</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>Description</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>Nil Rated Supplies</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>Exempted(other than nil rated/non GST supply)</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>Non-GST Supplies</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>Inter-State supplies to registered persons</t>
+        </is>
+      </c>
+      <c r="B5" t="n">
+        <v>21143</v>
+      </c>
+      <c r="C5" t="n">
+        <v>51235</v>
+      </c>
+      <c r="D5" t="n">
+        <v>5213</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>Intra-State supplies to registered persons</t>
+        </is>
+      </c>
+      <c r="B6" t="n">
+        <v>525</v>
+      </c>
+      <c r="C6" t="n">
+        <v>52135</v>
+      </c>
+      <c r="D6" t="n">
+        <v>5435</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>Inter-State supplies to unregistered persons</t>
+        </is>
+      </c>
+      <c r="B7" t="n">
+        <v>1234</v>
+      </c>
+      <c r="C7" t="n">
+        <v>512</v>
+      </c>
+      <c r="D7" t="n">
+        <v>5123</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>Intra-State supplies to unregistered persons</t>
+        </is>
+      </c>
+      <c r="B8" t="n">
+        <v>684</v>
+      </c>
+      <c r="C8" t="n">
+        <v>998</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet18.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:E9"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>Summary for doc_issue</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>Nature of Document</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>Sr. No. From</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>Sr. No. To</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>Total Number</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>Cancelled</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>Invoices for outward supply</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>INV-001</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>INV-100</t>
+        </is>
+      </c>
+      <c r="D5" t="n">
+        <v>100</v>
+      </c>
+      <c r="E5" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>Invoices for outward supply</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>INV-201</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>INV-250</t>
+        </is>
+      </c>
+      <c r="D6" t="n">
+        <v>50</v>
+      </c>
+      <c r="E6" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>Credit Note</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>CN-001</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>CN-010</t>
+        </is>
+      </c>
+      <c r="D7" t="n">
+        <v>10</v>
+      </c>
+      <c r="E7" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>Debit Note</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>DN-001</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>DN-005</t>
+        </is>
+      </c>
+      <c r="D8" t="n">
+        <v>5</v>
+      </c>
+      <c r="E8" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>Delivery Challan for job work</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>DC-001</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>DC-020</t>
+        </is>
+      </c>
+      <c r="D9" t="n">
+        <v>20</v>
+      </c>
+      <c r="E9" t="n">
+        <v>3</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet19.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
   <dimension ref="A1:K7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="inlineStr">
         <is>
-          <t>Summary for hsn(b2c)</t>
+          <t>Summary for hsn(b2b)</t>
         </is>
       </c>
     </row>
@@ -2468,6 +2653,183 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet20.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:K7"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>Summary for hsn(b2c)</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>HSN</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>Description</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>UQC</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>Total Quantity</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>Total Value</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>Rate</t>
+        </is>
+      </c>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>Taxable Value</t>
+        </is>
+      </c>
+      <c r="H4" t="inlineStr">
+        <is>
+          <t>Integrated Tax Amount</t>
+        </is>
+      </c>
+      <c r="I4" t="inlineStr">
+        <is>
+          <t>Central Tax Amount</t>
+        </is>
+      </c>
+      <c r="J4" t="inlineStr">
+        <is>
+          <t>State/UT Tax Amount</t>
+        </is>
+      </c>
+      <c r="K4" t="inlineStr">
+        <is>
+          <t>Cess Amount</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>0101</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>Live horses</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>NOS-NUMBERS</t>
+        </is>
+      </c>
+      <c r="D5" t="n">
+        <v>10</v>
+      </c>
+      <c r="E5" t="n">
+        <v>118000</v>
+      </c>
+      <c r="F5" t="n">
+        <v>18</v>
+      </c>
+      <c r="G5" t="n">
+        <v>100000</v>
+      </c>
+      <c r="H5" t="n">
+        <v>18000</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>0102</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>Live bovine animals</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>NOS-NUMBERS</t>
+        </is>
+      </c>
+      <c r="D6" t="n">
+        <v>5</v>
+      </c>
+      <c r="E6" t="n">
+        <v>52500</v>
+      </c>
+      <c r="F6" t="n">
+        <v>5</v>
+      </c>
+      <c r="G6" t="n">
+        <v>50000</v>
+      </c>
+      <c r="H6" t="n">
+        <v>2500</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>1006</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>Rice</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>KGS-KILOGRAMS</t>
+        </is>
+      </c>
+      <c r="D7" t="n">
+        <v>1000</v>
+      </c>
+      <c r="E7" t="n">
+        <v>105000</v>
+      </c>
+      <c r="F7" t="n">
+        <v>5</v>
+      </c>
+      <c r="G7" t="n">
+        <v>100000</v>
+      </c>
+      <c r="I7" t="n">
+        <v>2500</v>
+      </c>
+      <c r="J7" t="n">
+        <v>2500</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>

</xml_diff>

<commit_message>
feat(gstr1): e-commerce sections, completing all 30 worksheets
</commit_message>
<xml_diff>
--- a/fixtures/gstr1/demo-workbook.xlsx
+++ b/fixtures/gstr1/demo-workbook.xlsx
@@ -27,6 +27,16 @@
     <sheet name="docs" sheetId="18" state="visible" r:id="rId18"/>
     <sheet name="hsn(b2b)" sheetId="19" state="visible" r:id="rId19"/>
     <sheet name="hsn(b2c)" sheetId="20" state="visible" r:id="rId20"/>
+    <sheet name="eco" sheetId="21" state="visible" r:id="rId21"/>
+    <sheet name="ecoa" sheetId="22" state="visible" r:id="rId22"/>
+    <sheet name="ecob2b" sheetId="23" state="visible" r:id="rId23"/>
+    <sheet name="ecourp2b" sheetId="24" state="visible" r:id="rId24"/>
+    <sheet name="ecob2c" sheetId="25" state="visible" r:id="rId25"/>
+    <sheet name="ecourp2c" sheetId="26" state="visible" r:id="rId26"/>
+    <sheet name="ecoab2b" sheetId="27" state="visible" r:id="rId27"/>
+    <sheet name="ecoab2c" sheetId="28" state="visible" r:id="rId28"/>
+    <sheet name="ecoaurp2b" sheetId="29" state="visible" r:id="rId29"/>
+    <sheet name="ecoaurp2c" sheetId="30" state="visible" r:id="rId30"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -2830,6 +2840,1043 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet21.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:H6"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>Summary for eco</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>Nature of Supply</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>GSTIN of E-Commerce Operator</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>E-Commerce Operator Name</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>Net value of supplies</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>Integrated tax</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>Central tax</t>
+        </is>
+      </c>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>State/UT tax</t>
+        </is>
+      </c>
+      <c r="H4" t="inlineStr">
+        <is>
+          <t>Cess</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>Liable to collect tax u/s 52(TCS)</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>12AJIPA1572E1C7</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>Acme Marketplace</t>
+        </is>
+      </c>
+      <c r="D5" t="n">
+        <v>100000</v>
+      </c>
+      <c r="E5" t="n">
+        <v>18000</v>
+      </c>
+      <c r="F5" t="n">
+        <v>0</v>
+      </c>
+      <c r="G5" t="n">
+        <v>0</v>
+      </c>
+      <c r="H5" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>Liable to pay tax u/s 9(5)</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>12AJIPA1572E1C7</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>Acme Marketplace</t>
+        </is>
+      </c>
+      <c r="D6" t="n">
+        <v>50000</v>
+      </c>
+      <c r="E6" t="n">
+        <v>9000</v>
+      </c>
+      <c r="F6" t="n">
+        <v>0</v>
+      </c>
+      <c r="G6" t="n">
+        <v>0</v>
+      </c>
+      <c r="H6" t="n">
+        <v>0</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet22.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:K5"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>Summary for ecoa</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>Nature of Supply</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>Financial Year</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>Original Month/Quarter</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>Original GSTIN of E-Commerce Operator</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>Revised GSTIN of E-Commerce Operator</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>E-Commerce Operator Name</t>
+        </is>
+      </c>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>Revised Net value of supplies</t>
+        </is>
+      </c>
+      <c r="H4" t="inlineStr">
+        <is>
+          <t>Integrated tax</t>
+        </is>
+      </c>
+      <c r="I4" t="inlineStr">
+        <is>
+          <t>Central tax</t>
+        </is>
+      </c>
+      <c r="J4" t="inlineStr">
+        <is>
+          <t>State/UT tax</t>
+        </is>
+      </c>
+      <c r="K4" t="inlineStr">
+        <is>
+          <t>Cess</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>Liable to collect tax u/s 52(TCS)</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>2017-18</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>JULY</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>12AJIPA1572E1C7</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>12AJIPA1572E1C7</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>Acme Marketplace</t>
+        </is>
+      </c>
+      <c r="G5" t="n">
+        <v>120000</v>
+      </c>
+      <c r="H5" t="n">
+        <v>21600</v>
+      </c>
+      <c r="I5" t="n">
+        <v>0</v>
+      </c>
+      <c r="J5" t="n">
+        <v>0</v>
+      </c>
+      <c r="K5" t="n">
+        <v>0</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet23.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:L5"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>Summary for ecob2b</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>Supplier GSTIN/UIN</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>Supplier Name</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>Recipient GSTIN/UIN</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>Recipient Name</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>Document Number</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>Document Date</t>
+        </is>
+      </c>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>Value of supplies made</t>
+        </is>
+      </c>
+      <c r="H4" t="inlineStr">
+        <is>
+          <t>Place Of Supply</t>
+        </is>
+      </c>
+      <c r="I4" t="inlineStr">
+        <is>
+          <t>Document type</t>
+        </is>
+      </c>
+      <c r="J4" t="inlineStr">
+        <is>
+          <t>Rate</t>
+        </is>
+      </c>
+      <c r="K4" t="inlineStr">
+        <is>
+          <t>Taxable Value</t>
+        </is>
+      </c>
+      <c r="L4" t="inlineStr">
+        <is>
+          <t>Cess Amount</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>29AAPFU0939F1ZR</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>Seller Ltd</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>12GEOPS0823BBZH</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>Buyer Ltd</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>ECO-001</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>14-Jul-2017</t>
+        </is>
+      </c>
+      <c r="G5" t="n">
+        <v>118000</v>
+      </c>
+      <c r="H5" t="inlineStr">
+        <is>
+          <t>37-Andhra Pradesh</t>
+        </is>
+      </c>
+      <c r="I5" t="inlineStr">
+        <is>
+          <t>Invoice</t>
+        </is>
+      </c>
+      <c r="J5" t="n">
+        <v>18</v>
+      </c>
+      <c r="K5" t="n">
+        <v>100000</v>
+      </c>
+      <c r="L5" t="n">
+        <v>0</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet24.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:J5"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>Summary for ecourp2b</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>Recipient GSTIN/UIN</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>Recipient Name</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>Document Number</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>Document Date</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>Value of supplies made</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>Place Of Supply</t>
+        </is>
+      </c>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>Document type</t>
+        </is>
+      </c>
+      <c r="H4" t="inlineStr">
+        <is>
+          <t>Rate</t>
+        </is>
+      </c>
+      <c r="I4" t="inlineStr">
+        <is>
+          <t>Taxable Value</t>
+        </is>
+      </c>
+      <c r="J4" t="inlineStr">
+        <is>
+          <t>Cess Amount</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>12GEOPS0823BBZH</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>Buyer Ltd</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>ECO-002</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>15-Jul-2017</t>
+        </is>
+      </c>
+      <c r="E5" t="n">
+        <v>59000</v>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>37-Andhra Pradesh</t>
+        </is>
+      </c>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>Invoice</t>
+        </is>
+      </c>
+      <c r="H5" t="n">
+        <v>18</v>
+      </c>
+      <c r="I5" t="n">
+        <v>50000</v>
+      </c>
+      <c r="J5" t="n">
+        <v>0</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet25.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:F5"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>Summary for ecob2c</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>Supplier GSTIN/UIN</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>Supplier Name</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>Place Of Supply</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>Taxable Value</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>Rate</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>Cess Amount</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>29AAPFU0939F1ZR</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>Seller Ltd</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>37-Andhra Pradesh</t>
+        </is>
+      </c>
+      <c r="D5" t="n">
+        <v>50000</v>
+      </c>
+      <c r="E5" t="n">
+        <v>18</v>
+      </c>
+      <c r="F5" t="n">
+        <v>0</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet26.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:D5"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>Summary for ecourp2c</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>Place Of Supply</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>Taxable Value</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>Rate</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>Cess Amount</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>37-Andhra Pradesh</t>
+        </is>
+      </c>
+      <c r="B5" t="n">
+        <v>50000</v>
+      </c>
+      <c r="C5" t="n">
+        <v>18</v>
+      </c>
+      <c r="D5" t="n">
+        <v>0</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet27.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:N5"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>Summary for ecoab2b</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>Supplier GSTIN/UIN</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>Supplier Name</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>Recipient GSTIN/UIN</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>Recipient Name</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>Original Document Number</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>Original Document Date</t>
+        </is>
+      </c>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>Revised Document Number</t>
+        </is>
+      </c>
+      <c r="H4" t="inlineStr">
+        <is>
+          <t>Revised Document Date</t>
+        </is>
+      </c>
+      <c r="I4" t="inlineStr">
+        <is>
+          <t>Value of supplies made</t>
+        </is>
+      </c>
+      <c r="J4" t="inlineStr">
+        <is>
+          <t>Place Of Supply</t>
+        </is>
+      </c>
+      <c r="K4" t="inlineStr">
+        <is>
+          <t>Document type</t>
+        </is>
+      </c>
+      <c r="L4" t="inlineStr">
+        <is>
+          <t>Rate</t>
+        </is>
+      </c>
+      <c r="M4" t="inlineStr">
+        <is>
+          <t>Taxable Value</t>
+        </is>
+      </c>
+      <c r="N4" t="inlineStr">
+        <is>
+          <t>Cess Amount</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>29AAPFU0939F1ZR</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>Seller Ltd</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>12GEOPS0823BBZH</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>Buyer Ltd</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>ECO-001</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>14-Jul-2017</t>
+        </is>
+      </c>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>ECO-001-R</t>
+        </is>
+      </c>
+      <c r="H5" t="inlineStr">
+        <is>
+          <t>20-Jul-2017</t>
+        </is>
+      </c>
+      <c r="I5" t="n">
+        <v>118000</v>
+      </c>
+      <c r="J5" t="inlineStr">
+        <is>
+          <t>37-Andhra Pradesh</t>
+        </is>
+      </c>
+      <c r="K5" t="inlineStr">
+        <is>
+          <t>Invoice</t>
+        </is>
+      </c>
+      <c r="L5" t="n">
+        <v>18</v>
+      </c>
+      <c r="M5" t="n">
+        <v>100000</v>
+      </c>
+      <c r="N5" t="n">
+        <v>0</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet28.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:H5"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>Summary for ecoab2c</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>Financial Year</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>Original Month</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>Supplier GSTIN/UIN</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>Supplier Name</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>Place Of Supply</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>Rate</t>
+        </is>
+      </c>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>Taxable Value</t>
+        </is>
+      </c>
+      <c r="H4" t="inlineStr">
+        <is>
+          <t>Cess Amount</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>2017-18</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>JULY</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>29AAPFU0939F1ZR</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>Seller Ltd</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>37-Andhra Pradesh</t>
+        </is>
+      </c>
+      <c r="F5" t="n">
+        <v>18</v>
+      </c>
+      <c r="G5" t="n">
+        <v>50000</v>
+      </c>
+      <c r="H5" t="n">
+        <v>0</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet29.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:L5"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>Summary for ecoaurp2b</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>Recipient GSTIN/UIN</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>Recipient Name</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>Original Document Number</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>Original Document Date</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>Revised Document Number</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>Revised Document Date</t>
+        </is>
+      </c>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>Value of supplies made</t>
+        </is>
+      </c>
+      <c r="H4" t="inlineStr">
+        <is>
+          <t>Document type</t>
+        </is>
+      </c>
+      <c r="I4" t="inlineStr">
+        <is>
+          <t>Place Of Supply</t>
+        </is>
+      </c>
+      <c r="J4" t="inlineStr">
+        <is>
+          <t>Rate</t>
+        </is>
+      </c>
+      <c r="K4" t="inlineStr">
+        <is>
+          <t>Taxable Value</t>
+        </is>
+      </c>
+      <c r="L4" t="inlineStr">
+        <is>
+          <t>Cess Amount</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>12GEOPS0823BBZH</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>Buyer Ltd</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>ECO-002</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>15-Jul-2017</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>ECO-002-R</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>21-Jul-2017</t>
+        </is>
+      </c>
+      <c r="G5" t="n">
+        <v>59000</v>
+      </c>
+      <c r="H5" t="inlineStr">
+        <is>
+          <t>Invoice</t>
+        </is>
+      </c>
+      <c r="I5" t="inlineStr">
+        <is>
+          <t>37-Andhra Pradesh</t>
+        </is>
+      </c>
+      <c r="J5" t="n">
+        <v>18</v>
+      </c>
+      <c r="K5" t="n">
+        <v>50000</v>
+      </c>
+      <c r="L5" t="n">
+        <v>0</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
@@ -3027,6 +4074,85 @@
       </c>
       <c r="G9" t="n">
         <v>250000</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet30.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:F5"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>Summary for ecoaurp2c</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>Financial Year</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>Original Month</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>Place Of Supply</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>Rate</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>Taxable Value</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>Cess Amount</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>2017-18</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>JULY</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>37-Andhra Pradesh</t>
+        </is>
+      </c>
+      <c r="D5" t="n">
+        <v>18</v>
+      </c>
+      <c r="E5" t="n">
+        <v>50000</v>
+      </c>
+      <c r="F5" t="n">
+        <v>0</v>
       </c>
     </row>
   </sheetData>

</xml_diff>